<commit_message>
Wins Losses Update 2
</commit_message>
<xml_diff>
--- a/public/2024_2025 Bozo Bets.xlsx
+++ b/public/2024_2025 Bozo Bets.xlsx
@@ -17,168 +17,174 @@
     <t>Bozo Bet #1</t>
   </si>
   <si>
+    <t>NFL Side Bet #1</t>
+  </si>
+  <si>
+    <t>NFL Side Bet #2</t>
+  </si>
+  <si>
     <t>Bozo Bet #2</t>
   </si>
   <si>
     <t>Bozo Bet #3</t>
   </si>
   <si>
+    <t>NFL MNF Side Bet</t>
+  </si>
+  <si>
     <t>Bozo Bet #4</t>
   </si>
   <si>
+    <t>NFL Side Bet #3</t>
+  </si>
+  <si>
     <t>Bozo Bet #5</t>
   </si>
   <si>
-    <t>NFL Side Bet #1</t>
+    <t>NFL Side Bet #4</t>
+  </si>
+  <si>
+    <t>NFL Side Bet #5</t>
   </si>
   <si>
     <t>Bozo Bet #6</t>
   </si>
   <si>
+    <t>NFL Side Bet #6</t>
+  </si>
+  <si>
     <t>Bozo Bet #7</t>
   </si>
   <si>
-    <t>NFL Side Bet #2</t>
+    <t>NFL Side Bet #7</t>
   </si>
   <si>
     <t>Bozo Bet #8</t>
   </si>
   <si>
-    <t>NFL MNF Side Bet</t>
+    <t>Side Bet #8</t>
   </si>
   <si>
     <t>Bozo Bet #9</t>
   </si>
   <si>
+    <t>Side Bet #9</t>
+  </si>
+  <si>
     <t>Bozo Bet #10</t>
   </si>
   <si>
-    <t>NFL Side Bet #3</t>
+    <t>Side Bet #10</t>
   </si>
   <si>
     <t>Bozo Bet #11</t>
   </si>
   <si>
-    <t>NFL Side Bet #4</t>
+    <t>Side Bet #11</t>
   </si>
   <si>
     <t>Bozo Bet #12</t>
   </si>
   <si>
-    <t>NFL Side Bet #5</t>
-  </si>
-  <si>
     <t>Bozo Bet #13</t>
   </si>
   <si>
-    <t>NFL Side Bet #6</t>
+    <t>Wins/Losses</t>
   </si>
   <si>
     <t>Bozo Bet #14</t>
   </si>
   <si>
-    <t>NFL Side Bet #7</t>
-  </si>
-  <si>
     <t>Bozo Bet #15</t>
   </si>
   <si>
-    <t>Side Bet #8</t>
-  </si>
-  <si>
     <t>Bozo Bet #16</t>
   </si>
   <si>
-    <t>Side Bet #9</t>
-  </si>
-  <si>
     <t>Bozo Bet #17</t>
   </si>
   <si>
-    <t>Side Bet #10</t>
-  </si>
-  <si>
     <t>Bozo Bet #18</t>
   </si>
   <si>
-    <t>Side Bet #11</t>
-  </si>
-  <si>
-    <t>Wins/Losses</t>
+    <t>Sam</t>
   </si>
   <si>
     <t>Combined W/L</t>
   </si>
   <si>
-    <t>Sam</t>
+    <t>MHJ 70+ Yards</t>
   </si>
   <si>
     <t>KC ML</t>
   </si>
   <si>
+    <t>Diggs 50+ Yards</t>
+  </si>
+  <si>
     <t>Lamb 60/Nabers 50</t>
   </si>
   <si>
+    <t>Kelce O5.5 Rec</t>
+  </si>
+  <si>
+    <t>CIN ML</t>
+  </si>
+  <si>
     <t>USC -8</t>
   </si>
   <si>
-    <t>MHJ 70+ Yards</t>
+    <t>PHI +5.5</t>
   </si>
   <si>
     <t>NAVY -10.5</t>
   </si>
   <si>
-    <t>PHI +5.5</t>
+    <t>Dak/Burrow/Lamar 1+ TD Pass</t>
+  </si>
+  <si>
+    <t>Cousins 2+ Pass TDs</t>
   </si>
   <si>
     <t>OSU -3</t>
   </si>
   <si>
+    <t>Tua, Baker, CJ +1 TD passes</t>
+  </si>
+  <si>
     <t>PHI -3.5</t>
   </si>
   <si>
+    <t>AJ Brown 80+ Yards</t>
+  </si>
+  <si>
     <t>Texas -7.5</t>
   </si>
   <si>
-    <t>Diggs 50+ Yards</t>
+    <t>49ers ML</t>
   </si>
   <si>
     <t>Ohio State Buckeyes -6.5</t>
   </si>
   <si>
-    <t>Kelce O5.5 Rec</t>
+    <t>Lions of Detroit -4.5</t>
   </si>
   <si>
     <t>Notre Dame -3.5</t>
   </si>
   <si>
-    <t>CIN ML</t>
-  </si>
-  <si>
-    <t>49ers ML</t>
-  </si>
-  <si>
-    <t>Dak/Burrow/Lamar 1+ TD Pass</t>
+    <t>Joey B +275</t>
   </si>
   <si>
     <t>Eagles/Steelers O40</t>
   </si>
   <si>
-    <t>Cousins 2+ Pass TDs</t>
-  </si>
-  <si>
-    <t>Lions of Detroit -4.5</t>
-  </si>
-  <si>
-    <t>Tua, Baker, CJ +1 TD passes</t>
+    <t>8-4</t>
   </si>
   <si>
     <t>Ravens/Texans O44.5</t>
   </si>
   <si>
-    <t>AJ Brown 80+ Yards</t>
-  </si>
-  <si>
     <t>Texas -9.5</t>
   </si>
   <si>
@@ -188,76 +194,94 @@
     <t>Nico Collins 6 Receptions</t>
   </si>
   <si>
-    <t>Joey B +275</t>
-  </si>
-  <si>
     <t>Eagles ML/Eagles O22.5</t>
   </si>
   <si>
+    <t>Josh</t>
+  </si>
+  <si>
     <t>Saquon Anytime TD</t>
   </si>
   <si>
-    <t>8-4</t>
+    <t>GB ML</t>
+  </si>
+  <si>
+    <t>NO +5.5</t>
+  </si>
+  <si>
+    <t>LAC ML</t>
+  </si>
+  <si>
+    <t>WAS ML</t>
   </si>
   <si>
     <t>14-5</t>
   </si>
   <si>
-    <t>Josh</t>
-  </si>
-  <si>
-    <t>GB ML</t>
+    <t xml:space="preserve">Otton 5.5+ Receptions </t>
+  </si>
+  <si>
+    <t>GreenBay -4</t>
+  </si>
+  <si>
+    <t>Minn -3.5</t>
+  </si>
+  <si>
+    <t>Seattle+3</t>
+  </si>
+  <si>
+    <t>Bengals -1.5</t>
   </si>
   <si>
     <t>22-9</t>
   </si>
   <si>
-    <t>NO +5.5</t>
-  </si>
-  <si>
-    <t>LAC ML</t>
-  </si>
-  <si>
-    <t>WAS ML</t>
+    <t>6-3</t>
+  </si>
+  <si>
+    <t>Zach</t>
   </si>
   <si>
     <t>NYJ -1.5</t>
   </si>
   <si>
+    <t>PIT/IND U41</t>
+  </si>
+  <si>
     <t>DET +2.5</t>
   </si>
   <si>
-    <t xml:space="preserve">Otton 5.5+ Receptions </t>
-  </si>
-  <si>
-    <t>GreenBay -4</t>
-  </si>
-  <si>
-    <t>Minn -3.5</t>
+    <t>WAS/BAL O50.5</t>
+  </si>
+  <si>
+    <t>ATL ML</t>
   </si>
   <si>
     <t>Commanders ML</t>
   </si>
   <si>
-    <t>Seattle+3</t>
-  </si>
-  <si>
     <t>Texans ML</t>
   </si>
   <si>
+    <t>Broncos -5.5</t>
+  </si>
+  <si>
     <t>peeing on Kreitzer lawn - GreenBay -4</t>
   </si>
   <si>
-    <t>Bengals -1.5</t>
+    <t>Colts -2.5</t>
   </si>
   <si>
     <t>DET 1st Half -6.5</t>
   </si>
   <si>
+    <t>Raiders/Bucs over 46.5</t>
+  </si>
+  <si>
     <t>Alaba❌a -11.5</t>
   </si>
   <si>
-    <t>6-3</t>
+    <t>Ohio State ML</t>
   </si>
   <si>
     <t>Tyrone Tracy O 16.5 rec yards</t>
@@ -266,142 +290,166 @@
     <t>Notre Dame -4</t>
   </si>
   <si>
-    <t>Zach</t>
+    <t>5-3</t>
   </si>
   <si>
     <t>Penn State ML</t>
   </si>
   <si>
-    <t>PIT/IND U41</t>
+    <t>Jide</t>
   </si>
   <si>
     <t>Mahomes O 2.5 TDs</t>
   </si>
   <si>
-    <t>WAS/BAL O50.5</t>
-  </si>
-  <si>
-    <t>ATL ML</t>
-  </si>
-  <si>
-    <t>Broncos -5.5</t>
-  </si>
-  <si>
-    <t>Colts -2.5</t>
+    <t>NO ML</t>
+  </si>
+  <si>
+    <t>Kamara O25.5 RecYards</t>
+  </si>
+  <si>
+    <t>BAL ML</t>
+  </si>
+  <si>
+    <t>PIT ML</t>
+  </si>
+  <si>
+    <t>MIN ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cardinals +1 </t>
   </si>
   <si>
     <t>17-5</t>
   </si>
   <si>
-    <t>Raiders/Bucs over 46.5</t>
-  </si>
-  <si>
-    <t>Ohio State ML</t>
+    <t>KC Chiefs ML</t>
+  </si>
+  <si>
+    <t>5-2</t>
   </si>
   <si>
     <t>USC ML</t>
   </si>
   <si>
+    <t>Rick</t>
+  </si>
+  <si>
     <t>PIT/IND U40</t>
   </si>
   <si>
-    <t>5-3</t>
+    <t>WSH ML</t>
   </si>
   <si>
     <t>SMU +6.5</t>
   </si>
   <si>
+    <t>KC/NO O40.5</t>
+  </si>
+  <si>
     <t>ILL +4.5</t>
   </si>
   <si>
-    <t>Jide</t>
+    <t>BUF -2.5</t>
   </si>
   <si>
     <t>Illinois ML</t>
   </si>
   <si>
-    <t>NO ML</t>
+    <t>Nix O175 Pass Yards</t>
   </si>
   <si>
     <t>Colorado -3</t>
   </si>
   <si>
-    <t>Kamara O25.5 RecYards</t>
+    <t>Commanders -5.5</t>
   </si>
   <si>
     <t>Nebraska +9.5</t>
   </si>
   <si>
+    <t>Commanders -1</t>
+  </si>
+  <si>
     <t>TA&amp;M -2.5</t>
   </si>
   <si>
-    <t>BAL ML</t>
-  </si>
-  <si>
     <t>Syracuse +10.5</t>
   </si>
   <si>
-    <t>PIT ML</t>
-  </si>
-  <si>
-    <t>MIN ML</t>
+    <t xml:space="preserve"> Bengals -3</t>
   </si>
   <si>
     <t>SMU ML</t>
   </si>
   <si>
-    <t xml:space="preserve">Cardinals +1 </t>
-  </si>
-  <si>
     <t>Commanders -7.5 (-7.5)</t>
   </si>
   <si>
     <t>Clemson +12</t>
   </si>
   <si>
-    <t>KC Chiefs ML</t>
+    <t>OSU-Oregon O51.5</t>
+  </si>
+  <si>
+    <t>6-2</t>
+  </si>
+  <si>
+    <t>Shane</t>
+  </si>
+  <si>
+    <t>TB +5.5</t>
   </si>
   <si>
     <t>Seahawks -3.5</t>
   </si>
   <si>
-    <t>5-2</t>
+    <t>SEA -2.5</t>
+  </si>
+  <si>
+    <t>Worthy 40+ Yards</t>
   </si>
   <si>
     <t>Commanders/Bucs Over 50.5</t>
   </si>
   <si>
+    <t>BUF +4.5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mixon over 56.5 rushing </t>
   </si>
   <si>
-    <t>Rick</t>
+    <t>HOU ML</t>
   </si>
   <si>
     <t>Josh Allen rushing TD</t>
   </si>
   <si>
-    <t>WSH ML</t>
+    <t>CIN -3</t>
   </si>
   <si>
     <t>Saquan rushing Over</t>
   </si>
   <si>
-    <t>KC/NO O40.5</t>
-  </si>
-  <si>
-    <t>BUF -2.5</t>
+    <t>Josh Allen 200+ Pass Yards</t>
+  </si>
+  <si>
+    <t>Dolphins -3</t>
+  </si>
+  <si>
+    <t>Tampa Bay Bucs -2</t>
   </si>
   <si>
     <t>14-13</t>
   </si>
   <si>
-    <t>Nix O175 Pass Yards</t>
-  </si>
-  <si>
-    <t>Commanders -5.5</t>
-  </si>
-  <si>
-    <t>Commanders -1</t>
+    <t>Tampa Bay Bucs +2.5</t>
+  </si>
+  <si>
+    <t>Lions ML</t>
+  </si>
+  <si>
+    <t>9-2</t>
   </si>
   <si>
     <t>Kamara 25+ RecYards</t>
@@ -410,12 +458,21 @@
     <t>HOU +3.5</t>
   </si>
   <si>
-    <t xml:space="preserve"> Bengals -3</t>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Dalton 2+ TDs</t>
+  </si>
+  <si>
+    <t>BAL -2.5</t>
   </si>
   <si>
     <t>Vikings ML</t>
   </si>
   <si>
+    <t>Olave ATD</t>
+  </si>
+  <si>
     <t>Falcons ML</t>
   </si>
   <si>
@@ -425,210 +482,204 @@
     <t xml:space="preserve">Arizona Cardinals of the NFL +1 </t>
   </si>
   <si>
+    <t>Saints -6.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TJ Watt Over .25 sacks </t>
+  </si>
+  <si>
+    <t>Buccaneers -2.5</t>
+  </si>
+  <si>
+    <t>Seahawks ML</t>
+  </si>
+  <si>
+    <t>Buffalo Bills ML</t>
+  </si>
+  <si>
+    <t>LA rams ML</t>
+  </si>
+  <si>
+    <t>Dolphins -1.5</t>
+  </si>
+  <si>
+    <t>6-5</t>
+  </si>
+  <si>
+    <t>Matt</t>
+  </si>
+  <si>
+    <t>Mahomes ATD</t>
+  </si>
+  <si>
+    <t>PIT/LV O36.5</t>
+  </si>
+  <si>
+    <t>BUF ML</t>
+  </si>
+  <si>
+    <t>KC/TB O46</t>
+  </si>
+  <si>
+    <t>Saquon ATD</t>
+  </si>
+  <si>
+    <t>Houston texans ML</t>
+  </si>
+  <si>
+    <t>Philly Eagles -7</t>
+  </si>
+  <si>
+    <t>Arizona Cardinals ML</t>
+  </si>
+  <si>
+    <t>6-4</t>
+  </si>
+  <si>
+    <t>Ronnie</t>
+  </si>
+  <si>
+    <t>WAS/CHI O46</t>
+  </si>
+  <si>
+    <t>MIA +9.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Miami Dolphins -2.5 </t>
+  </si>
+  <si>
+    <t>Atlanta -6.5</t>
+  </si>
+  <si>
+    <t>2-2</t>
+  </si>
+  <si>
+    <t>Nate</t>
+  </si>
+  <si>
+    <t>CIN -4.5</t>
+  </si>
+  <si>
+    <t>IND +4</t>
+  </si>
+  <si>
+    <t>PHI -5.5</t>
+  </si>
+  <si>
+    <t>J Taylor O78.5 Yards</t>
+  </si>
+  <si>
+    <t>Lions -6.5</t>
+  </si>
+  <si>
+    <t>BenGals ML</t>
+  </si>
+  <si>
+    <t>Eagles -2.5</t>
+  </si>
+  <si>
+    <t>ND +4</t>
+  </si>
+  <si>
+    <t>Win $83.53</t>
+  </si>
+  <si>
     <t>Chargers ML</t>
   </si>
   <si>
-    <t>OSU-Oregon O51.5</t>
-  </si>
-  <si>
     <t>Mixon Anytime TD</t>
   </si>
   <si>
-    <t>6-2</t>
-  </si>
-  <si>
     <t>13-6</t>
   </si>
   <si>
-    <t>Shane</t>
-  </si>
-  <si>
-    <t>TB +5.5</t>
-  </si>
-  <si>
     <t>CSU -9</t>
   </si>
   <si>
-    <t>SEA -2.5</t>
-  </si>
-  <si>
     <t>MICH -7</t>
   </si>
   <si>
-    <t>Worthy 40+ Yards</t>
-  </si>
-  <si>
     <t>NC State -4.5</t>
   </si>
   <si>
-    <t>BUF +4.5</t>
-  </si>
-  <si>
     <t>TEM ML</t>
   </si>
   <si>
-    <t>HOU ML</t>
-  </si>
-  <si>
     <t>Utah St/WYO O54.5</t>
   </si>
   <si>
-    <t>CIN -3</t>
-  </si>
-  <si>
     <t>Army -19</t>
   </si>
   <si>
-    <t>Josh Allen 200+ Pass Yards</t>
-  </si>
-  <si>
     <t>BYU ML</t>
   </si>
   <si>
-    <t>Dolphins -3</t>
-  </si>
-  <si>
     <t>ND -17.5</t>
   </si>
   <si>
-    <t>Tampa Bay Bucs -2</t>
-  </si>
-  <si>
     <t>SMU -5.5</t>
   </si>
   <si>
-    <t>Tampa Bay Bucs +2.5</t>
-  </si>
-  <si>
     <t>SMU -8.5</t>
   </si>
   <si>
-    <t>Lions ML</t>
-  </si>
-  <si>
     <t>Louisiana -1</t>
   </si>
   <si>
-    <t>9-2</t>
-  </si>
-  <si>
     <t>Broncos ML</t>
   </si>
   <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Dalton 2+ TDs</t>
-  </si>
-  <si>
     <t>LAC-HOU O39.5</t>
   </si>
   <si>
-    <t>BAL -2.5</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Texans +11.5</t>
   </si>
   <si>
-    <t>Olave ATD</t>
-  </si>
-  <si>
-    <t>Saints -6.5</t>
-  </si>
-  <si>
     <t>Commanders +10.5</t>
   </si>
   <si>
-    <t xml:space="preserve">TJ Watt Over .25 sacks </t>
-  </si>
-  <si>
     <t>O40.5</t>
   </si>
   <si>
-    <t>Buccaneers -2.5</t>
-  </si>
-  <si>
-    <t>Seahawks ML</t>
-  </si>
-  <si>
     <t>18-8</t>
   </si>
   <si>
-    <t>Buffalo Bills ML</t>
-  </si>
-  <si>
-    <t>LA rams ML</t>
-  </si>
-  <si>
     <t>LAC +6.5</t>
   </si>
   <si>
-    <t>Dolphins -1.5</t>
-  </si>
-  <si>
     <t>DAL -1.5</t>
   </si>
   <si>
     <t>DAL +4.5</t>
   </si>
   <si>
-    <t>6-5</t>
-  </si>
-  <si>
     <t>BUF -3.5</t>
   </si>
   <si>
-    <t>Matt</t>
-  </si>
-  <si>
     <t>Bengals -3</t>
   </si>
   <si>
-    <t>Mahomes ATD</t>
-  </si>
-  <si>
     <t>49ers -2.5</t>
   </si>
   <si>
     <t>Dolphins -2.5</t>
   </si>
   <si>
-    <t>PIT/LV O36.5</t>
-  </si>
-  <si>
-    <t>BUF ML</t>
-  </si>
-  <si>
     <t>Lions -5.5</t>
   </si>
   <si>
-    <t>KC/TB O46</t>
-  </si>
-  <si>
     <t>Ohio State/Xichigan O37.5</t>
   </si>
   <si>
-    <t>Saquon ATD</t>
-  </si>
-  <si>
     <t>Bengals ML</t>
   </si>
   <si>
-    <t>Houston texans ML</t>
-  </si>
-  <si>
     <t>Steelers +7 (-312) it was -255 when I submitted the pick!</t>
   </si>
   <si>
-    <t>Philly Eagles -7</t>
-  </si>
-  <si>
     <t>Bills -3.5</t>
   </si>
   <si>
-    <t>Arizona Cardinals ML</t>
-  </si>
-  <si>
     <t>Bills +3.5</t>
   </si>
   <si>
@@ -641,33 +692,18 @@
     <t>23-7</t>
   </si>
   <si>
-    <t>6-4</t>
-  </si>
-  <si>
     <t>OK State +4.5</t>
   </si>
   <si>
-    <t>Ronnie</t>
-  </si>
-  <si>
     <t>MIA FL -4.5</t>
   </si>
   <si>
-    <t>WAS/CHI O46</t>
-  </si>
-  <si>
     <t>BYU +2.5</t>
   </si>
   <si>
-    <t>MIA +9.5</t>
-  </si>
-  <si>
     <t>Army/Air Force over 42</t>
   </si>
   <si>
-    <t xml:space="preserve">Miami Dolphins -2.5 </t>
-  </si>
-  <si>
     <t>Georgia ML</t>
   </si>
   <si>
@@ -680,57 +716,24 @@
     <t>Army -6</t>
   </si>
   <si>
-    <t>Atlanta -6.5</t>
-  </si>
-  <si>
-    <t>2-2</t>
-  </si>
-  <si>
     <t>chiefs -4</t>
   </si>
   <si>
-    <t>Nate</t>
-  </si>
-  <si>
-    <t>CIN -4.5</t>
-  </si>
-  <si>
-    <t>IND +4</t>
-  </si>
-  <si>
     <t>Jahmyr Gibbs anytime TD</t>
   </si>
   <si>
-    <t>PHI -5.5</t>
-  </si>
-  <si>
     <t>butker 2+ FG</t>
   </si>
   <si>
-    <t>J Taylor O78.5 Yards</t>
-  </si>
-  <si>
     <t>each team to score 1 rush and 1 passing td</t>
   </si>
   <si>
-    <t>Lions -6.5</t>
-  </si>
-  <si>
     <t>16-14</t>
   </si>
   <si>
-    <t>BenGals ML</t>
-  </si>
-  <si>
-    <t>Eagles -2.5</t>
-  </si>
-  <si>
     <t>PIT/LAC O36</t>
   </si>
   <si>
-    <t>ND +4</t>
-  </si>
-  <si>
     <t>OSU/MSU O48</t>
   </si>
   <si>
@@ -798,9 +801,6 @@
   </si>
   <si>
     <t>Colts -6.5</t>
-  </si>
-  <si>
-    <t>Win $83.53</t>
   </si>
   <si>
     <t xml:space="preserve">Saquan Anytime TD. </t>
@@ -913,14 +913,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
-        <bgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -949,10 +949,10 @@
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf quotePrefix="1" borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf quotePrefix="1" borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -964,10 +964,10 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -978,10 +978,10 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -1229,666 +1229,666 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
       <c r="W1" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G2" s="4" t="s">
+      <c r="C2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="E2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="N2" s="5" t="s">
+      <c r="G2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M2" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="N2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="O2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="P2" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="R2" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="Q2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="R2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="U2" s="6" t="s">
+      <c r="T2" s="5" t="s">
         <v>60</v>
       </c>
+      <c r="U2" s="7" t="s">
+        <v>62</v>
+      </c>
       <c r="V2" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="W2" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="X2" s="9" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="N3" s="5" t="s">
+      <c r="F3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="O3" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="U3" s="6" t="s">
-        <v>87</v>
+      <c r="J3" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="U3" s="7" t="s">
+        <v>95</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="W3" s="10">
         <v>46328.0</v>
       </c>
       <c r="X3" s="9" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="F4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q4" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="Q4" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="S4" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="T4" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="U4" s="6" t="s">
-        <v>123</v>
+      <c r="R4" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="U4" s="7" t="s">
+        <v>138</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="W4" s="10">
         <v>46275.0</v>
       </c>
       <c r="X4" s="9" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="S5" s="4" t="s">
-        <v>139</v>
+        <v>94</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>191</v>
       </c>
       <c r="V5" s="3" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="W5" s="10">
         <v>46238.0</v>
       </c>
       <c r="X5" s="9" t="s">
-        <v>141</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="N6" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="O6" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="Q6" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="R6" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="S6" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="T6" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="U6" s="6" t="s">
-        <v>176</v>
+        <v>106</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="T6" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="U6" s="7" t="s">
+        <v>208</v>
       </c>
       <c r="V6" s="3" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="W6" s="10">
         <v>46362.0</v>
       </c>
       <c r="X6" s="9" t="s">
-        <v>179</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="O7" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="Q7" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="R7" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="S7" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="T7" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="U7" s="6" t="s">
-        <v>207</v>
+        <v>127</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="U7" s="7" t="s">
+        <v>224</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="W7" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="X7" s="9" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="I8" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="P8" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="J8" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="P8" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="R8" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="S8" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="T8" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="U8" s="6" t="s">
-        <v>232</v>
+      <c r="Q8" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="R8" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="S8" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="T8" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="U8" s="7" t="s">
+        <v>237</v>
       </c>
       <c r="V8" s="3" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
       <c r="W8" s="10">
         <v>46304.0</v>
       </c>
       <c r="X8" s="9" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="C9" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="G9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="F9" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="J9" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="K9" s="4" t="s">
+      <c r="I9" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="J9" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="K9" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="M9" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="N9" s="4" t="s">
+      <c r="L9" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="O9" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="P9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="R9" s="4" t="s">
+      <c r="M9" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="N9" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="S9" s="4" t="s">
+      <c r="O9" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="P9" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q9" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="R9" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="T9" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="U9" s="6" t="s">
+      <c r="S9" s="5" t="s">
         <v>250</v>
       </c>
+      <c r="T9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>251</v>
+      </c>
       <c r="V9" s="3" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="W9" s="8" t="s">
-        <v>141</v>
+        <v>192</v>
       </c>
       <c r="X9" s="9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="E10" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="I10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="H10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="J10" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="L10" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="N10" s="4" t="s">
+      <c r="K10" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="O10" s="4" t="s">
+      <c r="L10" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="N10" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="P10" s="5" t="s">
+      <c r="O10" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="R10" s="5" t="s">
+      <c r="P10" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="R10" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="S10" s="4" t="s">
+      <c r="S10" s="5" t="s">
         <v>264</v>
       </c>
       <c r="V10" s="3" t="s">
-        <v>211</v>
+        <v>174</v>
       </c>
       <c r="W10" s="10">
         <v>46360.0</v>
@@ -1899,70 +1899,70 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="B11" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="K11" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="L11" s="4" t="s">
+      <c r="L11" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="N11" s="5" t="s">
+      <c r="N11" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="O11" s="4" t="s">
+      <c r="O11" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="P11" s="5" t="s">
+      <c r="P11" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="Q11" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="R11" s="4" t="s">
+      <c r="Q11" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="R11" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="S11" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="T11" s="4" t="s">
+      <c r="S11" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="T11" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="U11" s="6" t="s">
+      <c r="U11" s="7" t="s">
         <v>283</v>
       </c>
       <c r="V11" s="3" t="s">
-        <v>225</v>
+        <v>180</v>
       </c>
       <c r="W11" s="10">
         <v>46363.0</v>
@@ -1973,38 +1973,38 @@
     </row>
     <row r="12">
       <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="6"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="7"/>
     </row>
     <row r="13">
       <c r="A13" s="14"/>
       <c r="B13" s="16">
         <v>11000</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="7">
         <v>16000.0</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="7">
         <v>25000.0</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="7">
         <v>10000.0</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="7">
         <v>10000.0</v>
       </c>
       <c r="G13" s="16">
@@ -2013,16 +2013,16 @@
       <c r="H13" s="16">
         <v>5500</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="7">
         <v>6843.0</v>
       </c>
-      <c r="J13" s="6">
+      <c r="J13" s="7">
         <v>14000.0</v>
       </c>
-      <c r="P13" s="6">
+      <c r="P13" s="7">
         <v>25.0</v>
       </c>
-      <c r="Q13" s="6">
+      <c r="Q13" s="7">
         <v>25.0</v>
       </c>
     </row>
@@ -2055,10 +2055,10 @@
       <c r="J14" s="15">
         <v>50.0</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="7">
         <v>50.0</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="7">
         <v>50.0</v>
       </c>
       <c r="Q14" s="16">
@@ -2067,7 +2067,7 @@
     </row>
     <row r="15">
       <c r="A15" s="14"/>
-      <c r="B15" s="6"/>
+      <c r="B15" s="7"/>
       <c r="E15" s="17" t="s">
         <v>285</v>
       </c>
@@ -5059,43 +5059,43 @@
     <row r="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
@@ -5110,415 +5110,415 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="K2" s="4" t="s">
+      <c r="H2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="K2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="M2" s="4" t="s">
-        <v>58</v>
+      <c r="M2" s="5" t="s">
+        <v>53</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>61</v>
+        <v>31</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="F3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="L3" s="7"/>
+      <c r="M3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="L3" s="6"/>
-      <c r="M3" s="4" t="s">
-        <v>78</v>
-      </c>
       <c r="N3" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="O3" s="7" t="s">
-        <v>81</v>
+        <v>61</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="F4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L4" s="7"/>
+      <c r="M4" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="L4" s="6"/>
-      <c r="M4" s="4" t="s">
-        <v>94</v>
-      </c>
       <c r="N4" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="O4" s="7" t="s">
-        <v>97</v>
+        <v>75</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="I5" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="O5" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="K6" s="7"/>
+      <c r="L6" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="M6" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>138</v>
-      </c>
       <c r="N6" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>140</v>
+        <v>106</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B7" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="L7" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="M7" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="O7" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="L7" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="O7" s="7" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>180</v>
+        <v>148</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>160</v>
       </c>
       <c r="L8" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>183</v>
+        <v>161</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>162</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>186</v>
+        <v>148</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>202</v>
+        <v>164</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>171</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>204</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>74</v>
+        <v>172</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>81</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="O9" s="7" t="s">
-        <v>209</v>
+        <v>164</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>217</v>
+        <v>174</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>177</v>
       </c>
       <c r="L10" s="13"/>
-      <c r="M10" s="5" t="s">
-        <v>222</v>
+      <c r="M10" s="4" t="s">
+        <v>178</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="O10" s="7" t="s">
-        <v>223</v>
+        <v>174</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="L11" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>238</v>
+        <v>180</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>188</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="O11" s="7" t="s">
-        <v>81</v>
+        <v>180</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14"/>
-      <c r="B12" s="6">
+      <c r="B12" s="7">
         <v>5500.0</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="7">
         <v>17000.0</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="7">
         <v>1500.0</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="7">
         <v>1300.0</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="7">
         <v>3000.0</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="7">
         <v>10834.0</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="7">
         <v>2800.0</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I12" s="7">
         <v>5753.0</v>
       </c>
-      <c r="M12" s="6">
+      <c r="M12" s="7">
         <v>25.0</v>
       </c>
     </row>
@@ -5548,20 +5548,20 @@
       <c r="I13" s="15">
         <v>25.0</v>
       </c>
-      <c r="J13" s="6">
+      <c r="J13" s="7">
         <v>10.0</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="7">
         <v>10.0</v>
       </c>
-      <c r="M13" s="6">
+      <c r="M13" s="7">
         <v>9260.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14"/>
-      <c r="E14" s="4" t="s">
-        <v>262</v>
+      <c r="E14" s="5" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="15">

</xml_diff>